<commit_message>
Cap nhat du an 30/06/2026 10:59:15,16
</commit_message>
<xml_diff>
--- a/NOI DUNG LAM VIEC VOI AI.xlsx
+++ b/NOI DUNG LAM VIEC VOI AI.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1. WOKRS\1. THUY DIEN A LƯƠI\2- NHA MAY A LUOI\NAM 2026\3. P4\11. THEO DOI MANG XONG-OP DUONG HAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{22CCF0D2-E2BB-4AAA-8AC1-8E33DC4891FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC4CE148-A29F-4B05-9A45-0114BFAA1F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{3DE046CD-9242-4EBD-9D4C-DA3D99A3A767}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{3DE046CD-9242-4EBD-9D4C-DA3D99A3A767}"/>
   </bookViews>
   <sheets>
     <sheet name="Trang_tính1" sheetId="1" r:id="rId1"/>
+    <sheet name="Trang_tính2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,9 +40,41 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Bạn hãy thực hiện thiết kế bổ sung cho tôi tại sơ đồ tổng thể đường hầm, phần đoạn mô tà địa chất đứt gãy, bổ sung thêm tôi các đoạn lý trình như số liệu hình ảnh đính kèm. Bổ sung phần mô tả các đoạn địa chất đứt gãy bậc IV, các đoạn này được bố trí tương ứng với các lý trình và tỷ lệ đã mô tả trong dự án.  Các đoạn mô tả này được bôi màu đỏ. Rê chuột vào hiện thông tin từ lý trình nào đến lý trình nào. Nễu chưa rõ nhiệm vụ bạn hãy hỏi lại tôi để tránh làm không đứng ý ddood của tôi và sưa lại mất thời gian. Tôi cho phép bạn hỏi nhiều. Tôi không ngại bạn hỏi tôi nhiều nhé.</t>
+  </si>
+  <si>
+    <t>tôi có file cập nhập gits hup tôi mới đưa vào sự án. Bạn kiểm tra giúp tôi vi sao tôi cập nhập lên gits hup không được nhé. Nêu lý do vì sao và hiệu chỉnh để tôi cập nhập tự động. Chỉ cần nhấn vào file đó là tự đông comit lên ghithub. Nếu chưa rõ hỏi lại tôi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cập nhập cho tôi thêm nội dung các đường hàn (ĐH) có măng xồng (MX) được thực hiện lắp đặt năm 2022 vào dự án. Các đường hàn còn lại thuộc năm 2021. Bố trí thêm bảng tổng hợp tại tap thống kê đường hàn đã thực hiện MX năm 2021 và 2022. Đường hàn năm 2022 theo hình ảnh đính kèm. Chưa rõ mục đích, hay cần cụ thể chi tiết nào hỏi lại tôi. Càng nhiều câu hỏi càng tốt. </t>
+  </si>
+  <si>
+    <t>1. Hiện tại trong JSON, mỗi mục MX trong mo_ta_list chỉ là chuỗi như "ĐH-50.1-MX" — không có năm. Bạn muốn lưu năm theo: Gắn vào chuỗi: "ĐH-50.1-MX-2022
+2. nó là số thứ tự điểm đo trong .json
+3. Các đường hàn không có trong danh sách 2022 (hình ảnh) mà có -MX trong dữ liệu — tất cả đều là 2021
+4. Bảng tổng hợp MX theo năm bạn muốn hiển thị những cột Ví dụ: Năm | Số lượng MX | Danh sách ĐH. Sẽ xem sét hiệu chỉnh tiêp theo sau khi bạn đã thiết kế sơ bộ.
+5. Bảng tổng hợp này tính theo  theo từng phân đoạn (PĐ1 → PĐ6)
+6. Có cần hiển thị danh sách chi tiết từng ĐH-MX theo năm và cần đếm số lượng.
+7. Chỉ cần trong bản thống kê thôi.
+8. Tap thống kê tạm đặt cở phần đầu. rồi tính tiếp.</t>
+  </si>
+  <si>
+    <t>tôi muốn bổ sung sau: Khi rê chuột vào đường hàn (như anh đính kèm) thì sẽ hiện và bổ sung thêm thông tin là chỗ 3MX là như sau:
+"ĐH-33-MX [2021],
+ ĐH-33.1-MX [2021],
+ ĐH-33.2-MX [2021]"
+Nói chung cần cự thể rõ hơn chỗ chi tiết MX với dữ liệu đã có. Nếu chưa rõ họi lại chi tiết cho tôi.</t>
+  </si>
+  <si>
+    <t>Thao tác đong mở Public web trên githup</t>
+  </si>
+  <si>
+    <t>vào setting dự án</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kéo xuống dưới hiệu chỉnh </t>
   </si>
 </sst>
 </file>
@@ -78,10 +111,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -98,6 +135,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>72391</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>121919</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>4986925</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>3157770</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18635089-941C-2707-B258-B76800ABA13F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3013711" y="853439"/>
+          <a:ext cx="4912629" cy="3028231"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -417,21 +503,466 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F489D7E4-1B25-4FEF-99C4-9ED0C15B37EF}">
-  <dimension ref="A5:B5"/>
+  <dimension ref="A5:C129"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="113.625" customWidth="1"/>
+    <col min="3" max="3" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:2" ht="71.25" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="C5" s="2">
+        <v>46187</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="142.5" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="71.25" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" s="1"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" s="1"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12" s="1"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13" s="1"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" s="1"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>11</v>
+      </c>
+      <c r="B15" s="1"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B17" s="1"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B18" s="1"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B19" s="1"/>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B20" s="1"/>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B21" s="1"/>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B22" s="1"/>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B23" s="1"/>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B24" s="1"/>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B25" s="1"/>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B26" s="1"/>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B28" s="1"/>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B29" s="1"/>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B30" s="1"/>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B31" s="1"/>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B32" s="1"/>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B33" s="1"/>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B34" s="1"/>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B35" s="1"/>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B36" s="1"/>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B37" s="1"/>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B38" s="1"/>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B39" s="1"/>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B40" s="1"/>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B41" s="1"/>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B42" s="1"/>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B43" s="1"/>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B44" s="1"/>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B45" s="1"/>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B46" s="1"/>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B47" s="1"/>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B48" s="1"/>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B49" s="1"/>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B50" s="1"/>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B51" s="1"/>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B52" s="1"/>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B53" s="1"/>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B54" s="1"/>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B55" s="1"/>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B56" s="1"/>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B57" s="1"/>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B58" s="1"/>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B59" s="1"/>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B60" s="1"/>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B61" s="1"/>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B62" s="1"/>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B63" s="1"/>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B64" s="1"/>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B65" s="1"/>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B66" s="1"/>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B67" s="1"/>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B68" s="1"/>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B69" s="1"/>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B70" s="1"/>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B71" s="1"/>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B72" s="1"/>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B73" s="1"/>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B74" s="1"/>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B75" s="1"/>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B76" s="1"/>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B77" s="1"/>
+    </row>
+    <row r="78" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B78" s="1"/>
+    </row>
+    <row r="79" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B79" s="1"/>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B80" s="1"/>
+    </row>
+    <row r="81" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B81" s="1"/>
+    </row>
+    <row r="82" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B82" s="1"/>
+    </row>
+    <row r="83" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B83" s="1"/>
+    </row>
+    <row r="84" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B84" s="1"/>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B85" s="1"/>
+    </row>
+    <row r="86" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B86" s="1"/>
+    </row>
+    <row r="87" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B87" s="1"/>
+    </row>
+    <row r="88" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B88" s="1"/>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B89" s="1"/>
+    </row>
+    <row r="90" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B90" s="1"/>
+    </row>
+    <row r="91" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B91" s="1"/>
+    </row>
+    <row r="92" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B92" s="1"/>
+    </row>
+    <row r="93" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B93" s="1"/>
+    </row>
+    <row r="94" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B94" s="1"/>
+    </row>
+    <row r="95" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B95" s="1"/>
+    </row>
+    <row r="96" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B96" s="1"/>
+    </row>
+    <row r="97" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B97" s="1"/>
+    </row>
+    <row r="98" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B98" s="1"/>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B99" s="1"/>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B100" s="1"/>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B101" s="1"/>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B102" s="1"/>
+    </row>
+    <row r="103" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B103" s="1"/>
+    </row>
+    <row r="104" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B104" s="1"/>
+    </row>
+    <row r="105" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B105" s="1"/>
+    </row>
+    <row r="106" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B106" s="1"/>
+    </row>
+    <row r="107" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B107" s="1"/>
+    </row>
+    <row r="108" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B108" s="1"/>
+    </row>
+    <row r="109" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B109" s="1"/>
+    </row>
+    <row r="110" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B110" s="1"/>
+    </row>
+    <row r="111" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B111" s="1"/>
+    </row>
+    <row r="112" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B112" s="1"/>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B113" s="1"/>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B114" s="1"/>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B115" s="1"/>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B116" s="1"/>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B117" s="1"/>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B118" s="1"/>
+    </row>
+    <row r="119" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B119" s="1"/>
+    </row>
+    <row r="120" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B120" s="1"/>
+    </row>
+    <row r="121" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B121" s="1"/>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B122" s="1"/>
+    </row>
+    <row r="123" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B123" s="1"/>
+    </row>
+    <row r="124" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B124" s="1"/>
+    </row>
+    <row r="125" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B125" s="1"/>
+    </row>
+    <row r="126" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B126" s="1"/>
+    </row>
+    <row r="127" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B127" s="1"/>
+    </row>
+    <row r="128" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B128" s="1"/>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B129" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C80BD9E8-87B9-4402-B7D4-AA926BC240D7}">
+  <dimension ref="A2:A5"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22.25" style="3" customWidth="1"/>
+    <col min="2" max="2" width="67.5" style="3" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="249.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>